<commit_message>
Data base architecture done
</commit_message>
<xml_diff>
--- a/Progress/Roadmap_progress.xlsx
+++ b/Progress/Roadmap_progress.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1E8713-90C1-43D5-9BB9-79B2118EE9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
   </bookViews>
   <sheets>
     <sheet name="Road Map" sheetId="1" r:id="rId1"/>
@@ -877,15 +877,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -906,6 +897,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1224,21 +1224,21 @@
   <dimension ref="A1:E101"/>
   <sheetFormatPr defaultColWidth="57" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" style="8" customWidth="1"/>
     <col min="2" max="2" width="28.77734375" customWidth="1"/>
-    <col min="3" max="3" width="7" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="58.21875" customWidth="1"/>
     <col min="5" max="5" width="20.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -1252,7 +1252,7 @@
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="12" t="s">
         <v>29</v>
       </c>
       <c r="C2" s="4">
@@ -1269,7 +1269,7 @@
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="6"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="4">
         <v>2</v>
       </c>
@@ -1284,7 +1284,7 @@
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="6"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="4">
         <v>3</v>
       </c>
@@ -1299,7 +1299,7 @@
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="6"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="4">
         <v>4</v>
       </c>
@@ -1314,7 +1314,7 @@
       <c r="A6" s="4">
         <v>1</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="4">
         <v>5</v>
       </c>
@@ -1329,14 +1329,14 @@
       <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="4">
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1344,14 +1344,14 @@
       <c r="A8" s="4">
         <v>1</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="13"/>
       <c r="C8" s="4">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1359,14 +1359,14 @@
       <c r="A9" s="4">
         <v>1</v>
       </c>
-      <c r="B9" s="6"/>
+      <c r="B9" s="13"/>
       <c r="C9" s="4">
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1374,14 +1374,14 @@
       <c r="A10" s="4">
         <v>1</v>
       </c>
-      <c r="B10" s="6"/>
+      <c r="B10" s="13"/>
       <c r="C10" s="4">
         <v>9</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1389,14 +1389,14 @@
       <c r="A11" s="4">
         <v>1</v>
       </c>
-      <c r="B11" s="6"/>
+      <c r="B11" s="13"/>
       <c r="C11" s="4">
         <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1404,14 +1404,14 @@
       <c r="A12" s="4">
         <v>1</v>
       </c>
-      <c r="B12" s="6"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="4">
         <v>11</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1419,14 +1419,14 @@
       <c r="A13" s="4">
         <v>1</v>
       </c>
-      <c r="B13" s="6"/>
+      <c r="B13" s="13"/>
       <c r="C13" s="4">
         <v>12</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,14 +1434,14 @@
       <c r="A14" s="4">
         <v>1</v>
       </c>
-      <c r="B14" s="6"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="4">
         <v>13</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1449,14 +1449,14 @@
       <c r="A15" s="4">
         <v>1</v>
       </c>
-      <c r="B15" s="6"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="4">
         <v>14</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1464,14 +1464,14 @@
       <c r="A16" s="4">
         <v>1</v>
       </c>
-      <c r="B16" s="6"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="4">
         <v>15</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1479,14 +1479,14 @@
       <c r="A17" s="4">
         <v>1</v>
       </c>
-      <c r="B17" s="6"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="4">
         <v>16</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1494,14 +1494,14 @@
       <c r="A18" s="4">
         <v>1</v>
       </c>
-      <c r="B18" s="6"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="4">
         <v>17</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1509,14 +1509,14 @@
       <c r="A19" s="4">
         <v>1</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="4">
         <v>18</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1524,14 +1524,14 @@
       <c r="A20" s="4">
         <v>1</v>
       </c>
-      <c r="B20" s="6"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="4">
         <v>19</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1539,14 +1539,14 @@
       <c r="A21" s="4">
         <v>1</v>
       </c>
-      <c r="B21" s="6"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="4">
         <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1554,14 +1554,14 @@
       <c r="A22" s="4">
         <v>1</v>
       </c>
-      <c r="B22" s="6"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="4">
         <v>21</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1569,14 +1569,14 @@
       <c r="A23" s="4">
         <v>1</v>
       </c>
-      <c r="B23" s="7"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="4">
         <v>22</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="A24" s="4">
         <v>2</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="4">
@@ -1593,7 +1593,7 @@
       <c r="D24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       <c r="A25" s="4">
         <v>2</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="4">
@@ -1610,7 +1610,7 @@
       <c r="D25" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       <c r="A26" s="4">
         <v>2</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="4">
@@ -1627,7 +1627,7 @@
       <c r="D26" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       <c r="A27" s="4">
         <v>2</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C27" s="4">
@@ -1644,7 +1644,7 @@
       <c r="D27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       <c r="A28" s="4">
         <v>2</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C28" s="4">
@@ -1661,7 +1661,7 @@
       <c r="D28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1669,7 +1669,7 @@
       <c r="A29" s="4">
         <v>2</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C29" s="4">
@@ -1678,7 +1678,7 @@
       <c r="D29" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       <c r="A30" s="4">
         <v>2</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="4">
@@ -1695,7 +1695,7 @@
       <c r="D30" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       <c r="A31" s="4">
         <v>2</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C31" s="4">
@@ -1712,7 +1712,7 @@
       <c r="D31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       <c r="A32" s="4">
         <v>2</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C32" s="4">
@@ -1729,7 +1729,7 @@
       <c r="D32" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       <c r="A33" s="4">
         <v>2</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C33" s="4">
@@ -1746,7 +1746,7 @@
       <c r="D33" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       <c r="A34" s="4">
         <v>2</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C34" s="4">
@@ -1763,7 +1763,7 @@
       <c r="D34" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       <c r="A35" s="4">
         <v>2</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C35" s="4">
@@ -1780,7 +1780,7 @@
       <c r="D35" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E35" s="8" t="s">
+      <c r="E35" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       <c r="A36" s="4">
         <v>3</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="12" t="s">
         <v>45</v>
       </c>
       <c r="C36" s="4">
@@ -1797,7 +1797,7 @@
       <c r="D36" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1805,14 +1805,14 @@
       <c r="A37" s="4">
         <v>3</v>
       </c>
-      <c r="B37" s="6"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="4">
         <v>2</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1820,14 +1820,14 @@
       <c r="A38" s="4">
         <v>3</v>
       </c>
-      <c r="B38" s="6"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="4">
         <v>3</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1835,14 +1835,14 @@
       <c r="A39" s="4">
         <v>3</v>
       </c>
-      <c r="B39" s="6"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="4">
         <v>4</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E39" s="8" t="s">
+      <c r="E39" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1850,14 +1850,14 @@
       <c r="A40" s="4">
         <v>3</v>
       </c>
-      <c r="B40" s="6"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="4">
         <v>5</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="E40" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1865,14 +1865,14 @@
       <c r="A41" s="4">
         <v>3</v>
       </c>
-      <c r="B41" s="6"/>
+      <c r="B41" s="13"/>
       <c r="C41" s="4">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E41" s="8" t="s">
+      <c r="E41" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1880,14 +1880,14 @@
       <c r="A42" s="4">
         <v>3</v>
       </c>
-      <c r="B42" s="6"/>
+      <c r="B42" s="13"/>
       <c r="C42" s="4">
         <v>7</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1895,14 +1895,14 @@
       <c r="A43" s="4">
         <v>3</v>
       </c>
-      <c r="B43" s="6"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="4">
         <v>8</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E43" s="8" t="s">
+      <c r="E43" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1910,14 +1910,14 @@
       <c r="A44" s="4">
         <v>3</v>
       </c>
-      <c r="B44" s="6"/>
+      <c r="B44" s="13"/>
       <c r="C44" s="4">
         <v>9</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E44" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
       <c r="A45" s="4">
         <v>3</v>
       </c>
-      <c r="B45" s="6"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="4">
         <v>10</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E45" s="8" t="s">
+      <c r="E45" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1940,14 +1940,14 @@
       <c r="A46" s="4">
         <v>3</v>
       </c>
-      <c r="B46" s="6"/>
+      <c r="B46" s="13"/>
       <c r="C46" s="4">
         <v>11</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="E46" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1955,14 +1955,14 @@
       <c r="A47" s="4">
         <v>3</v>
       </c>
-      <c r="B47" s="6"/>
+      <c r="B47" s="13"/>
       <c r="C47" s="4">
         <v>12</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E47" s="8" t="s">
+      <c r="E47" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1970,14 +1970,14 @@
       <c r="A48" s="4">
         <v>3</v>
       </c>
-      <c r="B48" s="7"/>
+      <c r="B48" s="14"/>
       <c r="C48" s="4">
         <v>13</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E48" s="8" t="s">
+      <c r="E48" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       <c r="A49" s="4">
         <v>4</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="12" t="s">
         <v>59</v>
       </c>
       <c r="C49" s="4">
@@ -1994,7 +1994,7 @@
       <c r="D49" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2002,14 +2002,14 @@
       <c r="A50" s="4">
         <v>4</v>
       </c>
-      <c r="B50" s="6"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="4">
         <v>2</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E50" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2017,14 +2017,14 @@
       <c r="A51" s="4">
         <v>4</v>
       </c>
-      <c r="B51" s="6"/>
+      <c r="B51" s="13"/>
       <c r="C51" s="4">
         <v>3</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E51" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2032,14 +2032,14 @@
       <c r="A52" s="4">
         <v>4</v>
       </c>
-      <c r="B52" s="6"/>
+      <c r="B52" s="13"/>
       <c r="C52" s="4">
         <v>4</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E52" s="8" t="s">
+      <c r="E52" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2047,14 +2047,14 @@
       <c r="A53" s="4">
         <v>4</v>
       </c>
-      <c r="B53" s="6"/>
+      <c r="B53" s="13"/>
       <c r="C53" s="4">
         <v>5</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E53" s="8" t="s">
+      <c r="E53" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2062,14 +2062,14 @@
       <c r="A54" s="4">
         <v>4</v>
       </c>
-      <c r="B54" s="6"/>
+      <c r="B54" s="13"/>
       <c r="C54" s="4">
         <v>6</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E54" s="8" t="s">
+      <c r="E54" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2077,14 +2077,14 @@
       <c r="A55" s="4">
         <v>4</v>
       </c>
-      <c r="B55" s="6"/>
+      <c r="B55" s="13"/>
       <c r="C55" s="4">
         <v>7</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E55" s="8" t="s">
+      <c r="E55" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2092,14 +2092,14 @@
       <c r="A56" s="4">
         <v>4</v>
       </c>
-      <c r="B56" s="6"/>
+      <c r="B56" s="13"/>
       <c r="C56" s="4">
         <v>8</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E56" s="8" t="s">
+      <c r="E56" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2107,14 +2107,14 @@
       <c r="A57" s="4">
         <v>4</v>
       </c>
-      <c r="B57" s="6"/>
+      <c r="B57" s="13"/>
       <c r="C57" s="4">
         <v>9</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E57" s="8" t="s">
+      <c r="E57" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2122,14 +2122,14 @@
       <c r="A58" s="4">
         <v>4</v>
       </c>
-      <c r="B58" s="7"/>
+      <c r="B58" s="14"/>
       <c r="C58" s="4">
         <v>10</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E58" s="8" t="s">
+      <c r="E58" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       <c r="A59" s="4">
         <v>5</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="12" t="s">
         <v>69</v>
       </c>
       <c r="C59" s="4">
@@ -2146,7 +2146,7 @@
       <c r="D59" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E59" s="8" t="s">
+      <c r="E59" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2154,14 +2154,14 @@
       <c r="A60" s="4">
         <v>5</v>
       </c>
-      <c r="B60" s="6"/>
+      <c r="B60" s="13"/>
       <c r="C60" s="4">
         <v>2</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E60" s="8" t="s">
+      <c r="E60" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2169,14 +2169,14 @@
       <c r="A61" s="4">
         <v>5</v>
       </c>
-      <c r="B61" s="6"/>
+      <c r="B61" s="13"/>
       <c r="C61" s="4">
         <v>3</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E61" s="8" t="s">
+      <c r="E61" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2184,14 +2184,14 @@
       <c r="A62" s="4">
         <v>5</v>
       </c>
-      <c r="B62" s="6"/>
+      <c r="B62" s="13"/>
       <c r="C62" s="4">
         <v>4</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E62" s="8" t="s">
+      <c r="E62" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2199,14 +2199,14 @@
       <c r="A63" s="4">
         <v>5</v>
       </c>
-      <c r="B63" s="6"/>
+      <c r="B63" s="13"/>
       <c r="C63" s="4">
         <v>5</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E63" s="8" t="s">
+      <c r="E63" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2214,14 +2214,14 @@
       <c r="A64" s="4">
         <v>5</v>
       </c>
-      <c r="B64" s="6"/>
+      <c r="B64" s="13"/>
       <c r="C64" s="4">
         <v>6</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E64" s="8" t="s">
+      <c r="E64" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2229,14 +2229,14 @@
       <c r="A65" s="4">
         <v>5</v>
       </c>
-      <c r="B65" s="6"/>
+      <c r="B65" s="13"/>
       <c r="C65" s="4">
         <v>7</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E65" s="8" t="s">
+      <c r="E65" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2244,14 +2244,14 @@
       <c r="A66" s="4">
         <v>5</v>
       </c>
-      <c r="B66" s="6"/>
+      <c r="B66" s="13"/>
       <c r="C66" s="4">
         <v>8</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E66" s="8" t="s">
+      <c r="E66" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2259,14 +2259,14 @@
       <c r="A67" s="4">
         <v>5</v>
       </c>
-      <c r="B67" s="6"/>
+      <c r="B67" s="13"/>
       <c r="C67" s="4">
         <v>9</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E67" s="8" t="s">
+      <c r="E67" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2274,14 +2274,14 @@
       <c r="A68" s="4">
         <v>5</v>
       </c>
-      <c r="B68" s="7"/>
+      <c r="B68" s="14"/>
       <c r="C68" s="4">
         <v>10</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E68" s="8" t="s">
+      <c r="E68" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       <c r="A69" s="4">
         <v>6</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="12" t="s">
         <v>80</v>
       </c>
       <c r="C69" s="4">
@@ -2298,7 +2298,7 @@
       <c r="D69" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E69" s="8" t="s">
+      <c r="E69" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2306,14 +2306,14 @@
       <c r="A70" s="4">
         <v>6</v>
       </c>
-      <c r="B70" s="6"/>
+      <c r="B70" s="13"/>
       <c r="C70" s="4">
         <v>2</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E70" s="8" t="s">
+      <c r="E70" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2321,14 +2321,14 @@
       <c r="A71" s="4">
         <v>6</v>
       </c>
-      <c r="B71" s="6"/>
+      <c r="B71" s="13"/>
       <c r="C71" s="4">
         <v>3</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E71" s="8" t="s">
+      <c r="E71" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2336,14 +2336,14 @@
       <c r="A72" s="4">
         <v>6</v>
       </c>
-      <c r="B72" s="6"/>
+      <c r="B72" s="13"/>
       <c r="C72" s="4">
         <v>4</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E72" s="8" t="s">
+      <c r="E72" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2351,14 +2351,14 @@
       <c r="A73" s="4">
         <v>6</v>
       </c>
-      <c r="B73" s="6"/>
+      <c r="B73" s="13"/>
       <c r="C73" s="4">
         <v>5</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E73" s="8" t="s">
+      <c r="E73" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2366,14 +2366,14 @@
       <c r="A74" s="4">
         <v>6</v>
       </c>
-      <c r="B74" s="6"/>
+      <c r="B74" s="13"/>
       <c r="C74" s="4">
         <v>6</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E74" s="8" t="s">
+      <c r="E74" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2381,14 +2381,14 @@
       <c r="A75" s="4">
         <v>6</v>
       </c>
-      <c r="B75" s="6"/>
+      <c r="B75" s="13"/>
       <c r="C75" s="4">
         <v>7</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E75" s="8" t="s">
+      <c r="E75" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2396,14 +2396,14 @@
       <c r="A76" s="4">
         <v>6</v>
       </c>
-      <c r="B76" s="6"/>
+      <c r="B76" s="13"/>
       <c r="C76" s="4">
         <v>8</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E76" s="8" t="s">
+      <c r="E76" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2411,14 +2411,14 @@
       <c r="A77" s="4">
         <v>6</v>
       </c>
-      <c r="B77" s="6"/>
+      <c r="B77" s="13"/>
       <c r="C77" s="4">
         <v>9</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E77" s="8" t="s">
+      <c r="E77" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2426,14 +2426,14 @@
       <c r="A78" s="4">
         <v>6</v>
       </c>
-      <c r="B78" s="7"/>
+      <c r="B78" s="14"/>
       <c r="C78" s="4">
         <v>10</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E78" s="8" t="s">
+      <c r="E78" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       <c r="A79" s="4">
         <v>7</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="12" t="s">
         <v>91</v>
       </c>
       <c r="C79" s="4">
@@ -2450,7 +2450,7 @@
       <c r="D79" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E79" s="8" t="s">
+      <c r="E79" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2458,14 +2458,14 @@
       <c r="A80" s="4">
         <v>7</v>
       </c>
-      <c r="B80" s="6"/>
+      <c r="B80" s="13"/>
       <c r="C80" s="4">
         <v>2</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E80" s="8" t="s">
+      <c r="E80" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2473,14 +2473,14 @@
       <c r="A81" s="4">
         <v>7</v>
       </c>
-      <c r="B81" s="6"/>
+      <c r="B81" s="13"/>
       <c r="C81" s="4">
         <v>3</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E81" s="8" t="s">
+      <c r="E81" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2488,14 +2488,14 @@
       <c r="A82" s="4">
         <v>7</v>
       </c>
-      <c r="B82" s="6"/>
+      <c r="B82" s="13"/>
       <c r="C82" s="4">
         <v>4</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E82" s="8" t="s">
+      <c r="E82" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2503,14 +2503,14 @@
       <c r="A83" s="4">
         <v>7</v>
       </c>
-      <c r="B83" s="6"/>
+      <c r="B83" s="13"/>
       <c r="C83" s="4">
         <v>5</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E83" s="8" t="s">
+      <c r="E83" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2518,14 +2518,14 @@
       <c r="A84" s="4">
         <v>7</v>
       </c>
-      <c r="B84" s="6"/>
+      <c r="B84" s="13"/>
       <c r="C84" s="4">
         <v>6</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E84" s="8" t="s">
+      <c r="E84" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2533,14 +2533,14 @@
       <c r="A85" s="4">
         <v>7</v>
       </c>
-      <c r="B85" s="6"/>
+      <c r="B85" s="13"/>
       <c r="C85" s="4">
         <v>7</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E85" s="8" t="s">
+      <c r="E85" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2548,14 +2548,14 @@
       <c r="A86" s="4">
         <v>7</v>
       </c>
-      <c r="B86" s="6"/>
+      <c r="B86" s="13"/>
       <c r="C86" s="4">
         <v>8</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E86" s="8" t="s">
+      <c r="E86" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2563,14 +2563,14 @@
       <c r="A87" s="4">
         <v>7</v>
       </c>
-      <c r="B87" s="6"/>
+      <c r="B87" s="13"/>
       <c r="C87" s="4">
         <v>9</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E87" s="8" t="s">
+      <c r="E87" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2578,14 +2578,14 @@
       <c r="A88" s="4">
         <v>7</v>
       </c>
-      <c r="B88" s="6"/>
+      <c r="B88" s="13"/>
       <c r="C88" s="4">
         <v>10</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E88" s="8" t="s">
+      <c r="E88" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2593,14 +2593,14 @@
       <c r="A89" s="4">
         <v>7</v>
       </c>
-      <c r="B89" s="7"/>
+      <c r="B89" s="14"/>
       <c r="C89" s="4">
         <v>11</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E89" s="8" t="s">
+      <c r="E89" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       <c r="A90" s="4">
         <v>8</v>
       </c>
-      <c r="B90" s="5" t="s">
+      <c r="B90" s="12" t="s">
         <v>103</v>
       </c>
       <c r="C90" s="4">
@@ -2617,7 +2617,7 @@
       <c r="D90" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E90" s="8" t="s">
+      <c r="E90" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2625,14 +2625,14 @@
       <c r="A91" s="4">
         <v>8</v>
       </c>
-      <c r="B91" s="6"/>
+      <c r="B91" s="13"/>
       <c r="C91" s="4">
         <v>2</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E91" s="8" t="s">
+      <c r="E91" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2640,14 +2640,14 @@
       <c r="A92" s="4">
         <v>8</v>
       </c>
-      <c r="B92" s="6"/>
+      <c r="B92" s="13"/>
       <c r="C92" s="4">
         <v>3</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E92" s="8" t="s">
+      <c r="E92" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2655,14 +2655,14 @@
       <c r="A93" s="4">
         <v>8</v>
       </c>
-      <c r="B93" s="6"/>
+      <c r="B93" s="13"/>
       <c r="C93" s="4">
         <v>4</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E93" s="8" t="s">
+      <c r="E93" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2670,14 +2670,14 @@
       <c r="A94" s="4">
         <v>8</v>
       </c>
-      <c r="B94" s="6"/>
+      <c r="B94" s="13"/>
       <c r="C94" s="4">
         <v>5</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E94" s="8" t="s">
+      <c r="E94" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2685,14 +2685,14 @@
       <c r="A95" s="4">
         <v>8</v>
       </c>
-      <c r="B95" s="6"/>
+      <c r="B95" s="13"/>
       <c r="C95" s="4">
         <v>6</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E95" s="8" t="s">
+      <c r="E95" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2700,14 +2700,14 @@
       <c r="A96" s="4">
         <v>8</v>
       </c>
-      <c r="B96" s="6"/>
+      <c r="B96" s="13"/>
       <c r="C96" s="4">
         <v>7</v>
       </c>
       <c r="D96" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E96" s="8" t="s">
+      <c r="E96" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2715,14 +2715,14 @@
       <c r="A97" s="4">
         <v>8</v>
       </c>
-      <c r="B97" s="6"/>
+      <c r="B97" s="13"/>
       <c r="C97" s="4">
         <v>8</v>
       </c>
       <c r="D97" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="E97" s="8" t="s">
+      <c r="E97" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2730,14 +2730,14 @@
       <c r="A98" s="4">
         <v>8</v>
       </c>
-      <c r="B98" s="6"/>
+      <c r="B98" s="13"/>
       <c r="C98" s="4">
         <v>9</v>
       </c>
       <c r="D98" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E98" s="8" t="s">
+      <c r="E98" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2745,14 +2745,14 @@
       <c r="A99" s="4">
         <v>8</v>
       </c>
-      <c r="B99" s="6"/>
+      <c r="B99" s="13"/>
       <c r="C99" s="4">
         <v>10</v>
       </c>
       <c r="D99" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E99" s="8" t="s">
+      <c r="E99" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2760,14 +2760,14 @@
       <c r="A100" s="4">
         <v>8</v>
       </c>
-      <c r="B100" s="6"/>
+      <c r="B100" s="13"/>
       <c r="C100" s="4">
         <v>11</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E100" s="8" t="s">
+      <c r="E100" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2775,14 +2775,14 @@
       <c r="A101" s="4">
         <v>8</v>
       </c>
-      <c r="B101" s="7"/>
+      <c r="B101" s="14"/>
       <c r="C101" s="4">
         <v>12</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="E101" s="8" t="s">
+      <c r="E101" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2818,1133 +2818,1133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="11" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F2" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="13" t="s">
+      <c r="F2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F3" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="13" t="s">
+      <c r="F3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="F4" s="13" t="b">
+      <c r="F4" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G4" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="13" t="s">
+      <c r="G4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F5" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="13" t="s">
+      <c r="F5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="F6" s="13" t="b">
+      <c r="F6" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G6" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="13" t="b">
+      <c r="G6" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F7" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="13" t="s">
+      <c r="F7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="F8" s="13" t="b">
+      <c r="F8" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G8" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="13" t="b">
+      <c r="G8" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F9" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="13" t="s">
+      <c r="F9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="F10" s="13" t="b">
+      <c r="F10" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="13" t="b">
+      <c r="G10" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F11" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" s="13" t="s">
+      <c r="F11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="F12" s="13" t="b">
+      <c r="F12" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G12" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="13" t="b">
+      <c r="G12" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F13" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" s="13" t="s">
+      <c r="F13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="F14" s="13" t="b">
+      <c r="F14" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G14" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="13" t="b">
+      <c r="G14" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I15" s="13" t="s">
+      <c r="F15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="F16" s="13" t="b">
+      <c r="F16" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G16" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" s="13" t="b">
+      <c r="G16" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I16" s="13" t="s">
+      <c r="I16" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F17" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" s="13" t="s">
+      <c r="F17" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="F18" s="13" t="b">
+      <c r="F18" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G18" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" s="13" t="b">
+      <c r="G18" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I18" s="13" t="s">
+      <c r="I18" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="10" t="s">
         <v>172</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G19" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" s="13" t="s">
+      <c r="F19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="10" t="s">
         <v>174</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="F20" s="13" t="b">
+      <c r="F20" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G20" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" s="13" t="b">
+      <c r="G20" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I20" s="13" t="s">
+      <c r="I20" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G21" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" s="13" t="s">
+      <c r="F21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="10" t="s">
         <v>178</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="F22" s="13" t="b">
+      <c r="F22" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G22" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="13" t="b">
+      <c r="G22" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G23" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I23" s="13" t="s">
+      <c r="F23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="10" t="s">
         <v>183</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="10" t="s">
         <v>184</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="10" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="13" t="b">
+      <c r="F24" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G24" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" s="13" t="b">
+      <c r="G24" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H25" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" s="13" t="s">
+      <c r="F25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F26" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G26" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" s="13" t="b">
+      <c r="F26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I26" s="13" t="s">
+      <c r="I26" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="E27" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F27" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G27" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" s="13" t="b">
+      <c r="F27" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G27" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I27" s="13" t="s">
+      <c r="I27" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G28" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H28" s="13" t="b">
+      <c r="F28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G28" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="I28" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="10" t="s">
         <v>199</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C29" s="10" t="s">
         <v>202</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D29" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="E29" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F29" s="13" t="b">
+      <c r="F29" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G29" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="13" t="b">
+      <c r="G29" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="I29" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F30" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G30" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H30" s="13" t="b">
+      <c r="F30" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I30" s="13" t="s">
+      <c r="I30" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="10" t="s">
         <v>204</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="10" t="s">
         <v>207</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F31" s="13" t="b">
+      <c r="F31" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G31" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H31" s="13" t="b">
+      <c r="G31" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="I31" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="D32" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="E32" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F32" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G32" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H32" s="13" t="b">
+      <c r="F32" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I32" s="13" t="s">
+      <c r="I32" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="10" t="s">
         <v>213</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="D33" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="E33" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F33" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G33" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H33" s="13" t="b">
+      <c r="F33" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G33" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H33" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I33" s="13" t="s">
+      <c r="I33" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F34" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G34" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H34" s="13" t="b">
+      <c r="F34" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G34" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H34" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I34" s="13" t="s">
+      <c r="I34" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F35" s="13" t="b">
+      <c r="F35" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G35" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H35" s="13" t="b">
+      <c r="G35" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H35" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I35" s="13" t="s">
+      <c r="I35" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F36" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G36" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H36" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I36" s="13" t="s">
+      <c r="F36" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G36" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H36" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="10" t="s">
         <v>223</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B37" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F37" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G37" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H37" s="13" t="b">
+      <c r="F37" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G37" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H37" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I37" s="13" t="s">
+      <c r="I37" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="13" t="s">
+      <c r="A38" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="F38" s="13" t="b">
+      <c r="F38" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="G38" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H38" s="13" t="b">
+      <c r="G38" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H38" s="10" t="b">
         <v>0</v>
       </c>
-      <c r="I38" s="13" t="s">
+      <c r="I38" s="10" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="13" t="s">
+      <c r="A39" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="10" t="s">
         <v>229</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C39" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="D39" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="E39" s="13" t="s">
+      <c r="E39" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F39" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G39" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H39" s="13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I39" s="13" t="s">
+      <c r="F39" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G39" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H39" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I39" s="10" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
documented the redis architeture now will install the same via docker and used it
</commit_message>
<xml_diff>
--- a/Progress/Roadmap_progress.xlsx
+++ b/Progress/Roadmap_progress.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek\GIT Projects\MultiLinguinal_Application\Progress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1E8713-90C1-43D5-9BB9-79B2118EE9D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA07F8F-34B8-4F7E-9A73-55AD2DBEAD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
   </bookViews>
   <sheets>
     <sheet name="Road Map" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Road Map'!$A$1:$E$101</definedName>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="270">
   <si>
     <t>Step</t>
   </si>
@@ -731,6 +732,181 @@
   </si>
   <si>
     <t>संस्कृतम्</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Task Name</t>
+  </si>
+  <si>
+    <t>Requirements</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Languages</t>
+  </si>
+  <si>
+    <t>Users</t>
+  </si>
+  <si>
+    <t>Chat Rooms</t>
+  </si>
+  <si>
+    <t>Room Members</t>
+  </si>
+  <si>
+    <t>Messages</t>
+  </si>
+  <si>
+    <t>Translations</t>
+  </si>
+  <si>
+    <t>Message Status</t>
+  </si>
+  <si>
+    <t>Sessions</t>
+  </si>
+  <si>
+    <t>Attachments</t>
+  </si>
+  <si>
+    <t>Agent Executions</t>
+  </si>
+  <si>
+    <t>Tool Executions</t>
+  </si>
+  <si>
+    <t>Relationships/FKs</t>
+  </si>
+  <si>
+    <t>Constraints/Indexes</t>
+  </si>
+  <si>
+    <t>Lifecycle/Triggers</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>Data Integrity</t>
+  </si>
+  <si>
+    <t>Soft Delete/Retention</t>
+  </si>
+  <si>
+    <t>Audit/Compliance</t>
+  </si>
+  <si>
+    <t>Transactions</t>
+  </si>
+  <si>
+    <t>Concurrency</t>
+  </si>
+  <si>
+    <t>Query Design</t>
+  </si>
+  <si>
+    <t>Query Optimization</t>
+  </si>
+  <si>
+    <t>Database Testing</t>
+  </si>
+  <si>
+    <t>Migration Strategy</t>
+  </si>
+  <si>
+    <t>Backup/Recovery</t>
+  </si>
+  <si>
+    <t>Production Readiness</t>
+  </si>
+  <si>
+    <t>Who are the users were avail the access of tables and all so these can be park for now</t>
+  </si>
+  <si>
+    <t>| #  | Issue                                  | Solution                                                              | Layer      |
+| -- | -------------------------------------- | --------------------------------------------------------------------- | ---------- |
+| 1  | Deactivated user sending messages      | Backend checks account status before creating message                 | 🔵 Backend |
+| 2  | Deactivated room creator               | Backend prevents inactive user from creating rooms                    | 🔵 Backend |
+| 3  | Deactivated user remaining room member | Backend changes membership to `LEFT`/`REMOVED` during deactivation    | 🔵 Backend |
+| 4  | Message status user not in room        | Add composite FK/design relationship to enforce membership            | 🟢 DB      |
+| 5  | Attachment uploader not in room        | Backend validates uploader is a room member                           | 🔵 Backend |
+| 6  | Agent execution user/message mismatch  | Backend validates execution context                                   | 🔵 Backend |
+| 7  | Session lifecycle inconsistency        | Backend/scheduler manages expiration/revocation; DB checks timestamps | 🟡 Both    |
+| 8  | `DEACTIVATED` without `deactivated_at` | Add DB CHECK constraint                                               | 🟢 DB      |
+| 9  | Invalid deletion scheduling            | Add DB CHECK constraints for scheduling relationship                  | 🟢 DB      |
+| 10 | Deleted sender becoming NULL           | Keep `ON DELETE SET NULL`; this is intentional for message retention  | 🟢 DB      |</t>
+  </si>
+  <si>
+    <t>| Area                        | Decision                                                              |
+| --------------------------- | --------------------------------------------------------------------- |
+| **User account**            | Deactivate first, don't immediately delete                            |
+| **Deactivation timestamp**  | `deactivated_at` records when it happened                             |
+| **Deletion scheduling**     | `deletion_scheduled_at` determines when permanent deletion can happen |
+| **Sessions**                | Revoke sessions during deactivation                                   |
+| **Room membership**         | Mark membership `LEFT`/`REMOVED`, don't destroy history               |
+| **Messages**                | Preserve messages; use `is_deleted` for message deletion              |
+| **Attachments**             | Mark `DELETED`; physical storage cleanup handled separately           |
+| **Translations**            | Follow parent message retention                                       |
+| **Message status**          | Preserve required history                                             |
+| **Agent executions**        | Preserve execution/audit history                                      |
+| **Tool executions**         | Preserve execution/audit history                                      |
+| **Permanent user deletion** | Backend/scheduler performs it after retention period                  |
+| **Database cascading**      | Only use `CASCADE` where child data should genuinely disappear        |
+| **Retention cleanup**       | Backend scheduler/job, not PostgreSQL trigger                         |</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Created audit logs where all the logs will be captured</t>
+  </si>
+  <si>
+    <t>No changes required</t>
+  </si>
+  <si>
+    <t>Select query for all the tables</t>
+  </si>
+  <si>
+    <t>Absolutely. Let's do it from the beginning with no alternatives. Run these commands one by one in PowerShell.
+Step 1 — Remove the old backup
+Remove-Item .\backup.dump -ErrorAction SilentlyContinue
+Step 2 — Create the backup
+docker exec chat_application_DB pg_dump -U chat_app -d chat_app_db -p 32031 -Fc -f /tmp/backup.dump
+Step 3 — Copy the backup from Docker to your Windows folder
+docker cp chat_application_DB:/tmp/backup.dump .\backup.dump
+Step 4 — Check the backup file
+Get-Item .\backup.dump | Select-Object Name,Length
+You should see something like:
+Name          Length
+----          ------
+backup.dump   12345
+The exact size doesn't matter; Length must be greater than 0.
+Step 5 — Create a test restore database
+docker exec chat_application_DB dropdb -U chat_app -p 32031 --if-exists restore_db
+Then:
+docker exec chat_application_DB createdb -U chat_app -p 32031 restore_db
+Step 6 — Copy the backup back into Docker
+docker cp .\backup.dump chat_application_DB:/tmp/restore_backup.dump
+Step 7 — Restore
+docker exec chat_application_DB pg_restore -U chat_app -p 32031 -d restore_db /tmp/restore_backup.dump
+There should be no input file does not appear to be a valid archive error.
+Step 8 — Verify the restored database
+docker exec -it chat_application_DB psql -U chat_app -p 32031 -d restore_db
+Now inside PostgreSQL run:
+SELECT COUNT(*) FROM chat_app.users;
+Then:
+SELECT COUNT(*) FROM chat_app.language_configurations;
+Then:
+SELECT COUNT(*) FROM chat_app.messages;
+Exit:
+\q</t>
   </si>
 </sst>
 </file>
@@ -863,7 +1039,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -906,6 +1082,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2799,6 +2984,7 @@
     <mergeCell ref="B59:B68"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3951,4 +4137,387 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E8FE01D-536D-48C9-A873-39ECCBD84B79}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" style="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="149.33203125" style="15" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="17">
+        <v>6.1</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D2" s="17"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="17">
+        <v>6.2</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D3" s="17"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="17">
+        <v>6.3</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" s="17"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="17">
+        <v>6.4</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D5" s="17"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="17">
+        <v>6.5</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="17"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="17">
+        <v>6.6</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D7" s="17"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="17">
+        <v>6.7</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" s="17"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="17">
+        <v>6.8</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D9" s="17"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="17">
+        <v>6.9</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D10" s="17"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="17">
+        <v>6.1</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D11" s="17"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="17">
+        <v>6.11</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D12" s="17"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="17">
+        <v>6.12</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D13" s="17"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="17">
+        <v>6.13</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D14" s="17"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="17">
+        <v>6.14</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D15" s="17"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="17">
+        <v>6.15</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D16" s="17"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="17">
+        <v>6.16</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D17" s="17"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="17">
+        <v>6.17</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="17">
+        <v>6.18</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>251</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="17">
+        <v>6.19</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>252</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="17">
+        <v>6.2</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="17">
+        <v>6.21</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="17">
+        <v>6.22</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="17">
+        <v>6.23</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>256</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="17">
+        <v>6.24</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D25" s="17"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="17">
+        <v>6.25</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D26" s="17"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="17">
+        <v>6.26</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="17"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="17">
+        <v>6.27</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="17">
+        <v>6.28</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D29" s="17"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
commit changes to the main branch for redis implementation will start
</commit_message>
<xml_diff>
--- a/Progress/Roadmap_progress.xlsx
+++ b/Progress/Roadmap_progress.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek\GIT Projects\MultiLinguinal_Application\Progress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA07F8F-34B8-4F7E-9A73-55AD2DBEAD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF8D002-30BD-4D82-AB2A-0998B60DE824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
   </bookViews>
   <sheets>
     <sheet name="Road Map" sheetId="1" r:id="rId1"/>
@@ -1074,6 +1074,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1082,15 +1091,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1437,7 +1437,7 @@
       <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C2" s="4">
@@ -1454,7 +1454,7 @@
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="13"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4">
         <v>2</v>
       </c>
@@ -1469,7 +1469,7 @@
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="13"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4">
         <v>3</v>
       </c>
@@ -1484,7 +1484,7 @@
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="4">
         <v>4</v>
       </c>
@@ -1499,7 +1499,7 @@
       <c r="A6" s="4">
         <v>1</v>
       </c>
-      <c r="B6" s="13"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="4">
         <v>5</v>
       </c>
@@ -1514,37 +1514,37 @@
       <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="13"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="4">
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>31</v>
+      <c r="E7" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>1</v>
       </c>
-      <c r="B8" s="13"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="4">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>10</v>
+      <c r="E8" s="6" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>1</v>
       </c>
-      <c r="B9" s="13"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="4">
         <v>8</v>
       </c>
@@ -1559,7 +1559,7 @@
       <c r="A10" s="4">
         <v>1</v>
       </c>
-      <c r="B10" s="13"/>
+      <c r="B10" s="16"/>
       <c r="C10" s="4">
         <v>9</v>
       </c>
@@ -1574,7 +1574,7 @@
       <c r="A11" s="4">
         <v>1</v>
       </c>
-      <c r="B11" s="13"/>
+      <c r="B11" s="16"/>
       <c r="C11" s="4">
         <v>10</v>
       </c>
@@ -1589,7 +1589,7 @@
       <c r="A12" s="4">
         <v>1</v>
       </c>
-      <c r="B12" s="13"/>
+      <c r="B12" s="16"/>
       <c r="C12" s="4">
         <v>11</v>
       </c>
@@ -1604,7 +1604,7 @@
       <c r="A13" s="4">
         <v>1</v>
       </c>
-      <c r="B13" s="13"/>
+      <c r="B13" s="16"/>
       <c r="C13" s="4">
         <v>12</v>
       </c>
@@ -1619,7 +1619,7 @@
       <c r="A14" s="4">
         <v>1</v>
       </c>
-      <c r="B14" s="13"/>
+      <c r="B14" s="16"/>
       <c r="C14" s="4">
         <v>13</v>
       </c>
@@ -1634,7 +1634,7 @@
       <c r="A15" s="4">
         <v>1</v>
       </c>
-      <c r="B15" s="13"/>
+      <c r="B15" s="16"/>
       <c r="C15" s="4">
         <v>14</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="A16" s="4">
         <v>1</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="4">
         <v>15</v>
       </c>
@@ -1664,7 +1664,7 @@
       <c r="A17" s="4">
         <v>1</v>
       </c>
-      <c r="B17" s="13"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="4">
         <v>16</v>
       </c>
@@ -1679,7 +1679,7 @@
       <c r="A18" s="4">
         <v>1</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="4">
         <v>17</v>
       </c>
@@ -1694,7 +1694,7 @@
       <c r="A19" s="4">
         <v>1</v>
       </c>
-      <c r="B19" s="13"/>
+      <c r="B19" s="16"/>
       <c r="C19" s="4">
         <v>18</v>
       </c>
@@ -1709,7 +1709,7 @@
       <c r="A20" s="4">
         <v>1</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="16"/>
       <c r="C20" s="4">
         <v>19</v>
       </c>
@@ -1724,7 +1724,7 @@
       <c r="A21" s="4">
         <v>1</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="16"/>
       <c r="C21" s="4">
         <v>20</v>
       </c>
@@ -1739,7 +1739,7 @@
       <c r="A22" s="4">
         <v>1</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="16"/>
       <c r="C22" s="4">
         <v>21</v>
       </c>
@@ -1754,7 +1754,7 @@
       <c r="A23" s="4">
         <v>1</v>
       </c>
-      <c r="B23" s="14"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="4">
         <v>22</v>
       </c>
@@ -1769,7 +1769,7 @@
       <c r="A24" s="4">
         <v>2</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="15" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="4">
@@ -1786,7 +1786,7 @@
       <c r="A25" s="4">
         <v>2</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="4">
@@ -1803,7 +1803,7 @@
       <c r="A26" s="4">
         <v>2</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="4">
@@ -1820,7 +1820,7 @@
       <c r="A27" s="4">
         <v>2</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C27" s="4">
@@ -1837,7 +1837,7 @@
       <c r="A28" s="4">
         <v>2</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C28" s="4">
@@ -1854,7 +1854,7 @@
       <c r="A29" s="4">
         <v>2</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C29" s="4">
@@ -1871,7 +1871,7 @@
       <c r="A30" s="4">
         <v>2</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="4">
@@ -1888,7 +1888,7 @@
       <c r="A31" s="4">
         <v>2</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C31" s="4">
@@ -1905,7 +1905,7 @@
       <c r="A32" s="4">
         <v>2</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C32" s="4">
@@ -1922,7 +1922,7 @@
       <c r="A33" s="4">
         <v>2</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C33" s="4">
@@ -1939,7 +1939,7 @@
       <c r="A34" s="4">
         <v>2</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C34" s="4">
@@ -1956,7 +1956,7 @@
       <c r="A35" s="4">
         <v>2</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C35" s="4">
@@ -1973,7 +1973,7 @@
       <c r="A36" s="4">
         <v>3</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="15" t="s">
         <v>45</v>
       </c>
       <c r="C36" s="4">
@@ -1990,7 +1990,7 @@
       <c r="A37" s="4">
         <v>3</v>
       </c>
-      <c r="B37" s="13"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="4">
         <v>2</v>
       </c>
@@ -2005,7 +2005,7 @@
       <c r="A38" s="4">
         <v>3</v>
       </c>
-      <c r="B38" s="13"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="4">
         <v>3</v>
       </c>
@@ -2020,7 +2020,7 @@
       <c r="A39" s="4">
         <v>3</v>
       </c>
-      <c r="B39" s="13"/>
+      <c r="B39" s="16"/>
       <c r="C39" s="4">
         <v>4</v>
       </c>
@@ -2035,7 +2035,7 @@
       <c r="A40" s="4">
         <v>3</v>
       </c>
-      <c r="B40" s="13"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="4">
         <v>5</v>
       </c>
@@ -2050,7 +2050,7 @@
       <c r="A41" s="4">
         <v>3</v>
       </c>
-      <c r="B41" s="13"/>
+      <c r="B41" s="16"/>
       <c r="C41" s="4">
         <v>6</v>
       </c>
@@ -2065,7 +2065,7 @@
       <c r="A42" s="4">
         <v>3</v>
       </c>
-      <c r="B42" s="13"/>
+      <c r="B42" s="16"/>
       <c r="C42" s="4">
         <v>7</v>
       </c>
@@ -2080,7 +2080,7 @@
       <c r="A43" s="4">
         <v>3</v>
       </c>
-      <c r="B43" s="13"/>
+      <c r="B43" s="16"/>
       <c r="C43" s="4">
         <v>8</v>
       </c>
@@ -2095,7 +2095,7 @@
       <c r="A44" s="4">
         <v>3</v>
       </c>
-      <c r="B44" s="13"/>
+      <c r="B44" s="16"/>
       <c r="C44" s="4">
         <v>9</v>
       </c>
@@ -2110,7 +2110,7 @@
       <c r="A45" s="4">
         <v>3</v>
       </c>
-      <c r="B45" s="13"/>
+      <c r="B45" s="16"/>
       <c r="C45" s="4">
         <v>10</v>
       </c>
@@ -2125,7 +2125,7 @@
       <c r="A46" s="4">
         <v>3</v>
       </c>
-      <c r="B46" s="13"/>
+      <c r="B46" s="16"/>
       <c r="C46" s="4">
         <v>11</v>
       </c>
@@ -2140,7 +2140,7 @@
       <c r="A47" s="4">
         <v>3</v>
       </c>
-      <c r="B47" s="13"/>
+      <c r="B47" s="16"/>
       <c r="C47" s="4">
         <v>12</v>
       </c>
@@ -2155,7 +2155,7 @@
       <c r="A48" s="4">
         <v>3</v>
       </c>
-      <c r="B48" s="14"/>
+      <c r="B48" s="17"/>
       <c r="C48" s="4">
         <v>13</v>
       </c>
@@ -2170,7 +2170,7 @@
       <c r="A49" s="4">
         <v>4</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B49" s="15" t="s">
         <v>59</v>
       </c>
       <c r="C49" s="4">
@@ -2187,7 +2187,7 @@
       <c r="A50" s="4">
         <v>4</v>
       </c>
-      <c r="B50" s="13"/>
+      <c r="B50" s="16"/>
       <c r="C50" s="4">
         <v>2</v>
       </c>
@@ -2202,7 +2202,7 @@
       <c r="A51" s="4">
         <v>4</v>
       </c>
-      <c r="B51" s="13"/>
+      <c r="B51" s="16"/>
       <c r="C51" s="4">
         <v>3</v>
       </c>
@@ -2217,7 +2217,7 @@
       <c r="A52" s="4">
         <v>4</v>
       </c>
-      <c r="B52" s="13"/>
+      <c r="B52" s="16"/>
       <c r="C52" s="4">
         <v>4</v>
       </c>
@@ -2232,7 +2232,7 @@
       <c r="A53" s="4">
         <v>4</v>
       </c>
-      <c r="B53" s="13"/>
+      <c r="B53" s="16"/>
       <c r="C53" s="4">
         <v>5</v>
       </c>
@@ -2247,7 +2247,7 @@
       <c r="A54" s="4">
         <v>4</v>
       </c>
-      <c r="B54" s="13"/>
+      <c r="B54" s="16"/>
       <c r="C54" s="4">
         <v>6</v>
       </c>
@@ -2262,7 +2262,7 @@
       <c r="A55" s="4">
         <v>4</v>
       </c>
-      <c r="B55" s="13"/>
+      <c r="B55" s="16"/>
       <c r="C55" s="4">
         <v>7</v>
       </c>
@@ -2277,7 +2277,7 @@
       <c r="A56" s="4">
         <v>4</v>
       </c>
-      <c r="B56" s="13"/>
+      <c r="B56" s="16"/>
       <c r="C56" s="4">
         <v>8</v>
       </c>
@@ -2292,7 +2292,7 @@
       <c r="A57" s="4">
         <v>4</v>
       </c>
-      <c r="B57" s="13"/>
+      <c r="B57" s="16"/>
       <c r="C57" s="4">
         <v>9</v>
       </c>
@@ -2307,7 +2307,7 @@
       <c r="A58" s="4">
         <v>4</v>
       </c>
-      <c r="B58" s="14"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="4">
         <v>10</v>
       </c>
@@ -2322,7 +2322,7 @@
       <c r="A59" s="4">
         <v>5</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="15" t="s">
         <v>69</v>
       </c>
       <c r="C59" s="4">
@@ -2339,7 +2339,7 @@
       <c r="A60" s="4">
         <v>5</v>
       </c>
-      <c r="B60" s="13"/>
+      <c r="B60" s="16"/>
       <c r="C60" s="4">
         <v>2</v>
       </c>
@@ -2354,7 +2354,7 @@
       <c r="A61" s="4">
         <v>5</v>
       </c>
-      <c r="B61" s="13"/>
+      <c r="B61" s="16"/>
       <c r="C61" s="4">
         <v>3</v>
       </c>
@@ -2369,7 +2369,7 @@
       <c r="A62" s="4">
         <v>5</v>
       </c>
-      <c r="B62" s="13"/>
+      <c r="B62" s="16"/>
       <c r="C62" s="4">
         <v>4</v>
       </c>
@@ -2384,7 +2384,7 @@
       <c r="A63" s="4">
         <v>5</v>
       </c>
-      <c r="B63" s="13"/>
+      <c r="B63" s="16"/>
       <c r="C63" s="4">
         <v>5</v>
       </c>
@@ -2399,7 +2399,7 @@
       <c r="A64" s="4">
         <v>5</v>
       </c>
-      <c r="B64" s="13"/>
+      <c r="B64" s="16"/>
       <c r="C64" s="4">
         <v>6</v>
       </c>
@@ -2414,7 +2414,7 @@
       <c r="A65" s="4">
         <v>5</v>
       </c>
-      <c r="B65" s="13"/>
+      <c r="B65" s="16"/>
       <c r="C65" s="4">
         <v>7</v>
       </c>
@@ -2429,7 +2429,7 @@
       <c r="A66" s="4">
         <v>5</v>
       </c>
-      <c r="B66" s="13"/>
+      <c r="B66" s="16"/>
       <c r="C66" s="4">
         <v>8</v>
       </c>
@@ -2444,7 +2444,7 @@
       <c r="A67" s="4">
         <v>5</v>
       </c>
-      <c r="B67" s="13"/>
+      <c r="B67" s="16"/>
       <c r="C67" s="4">
         <v>9</v>
       </c>
@@ -2459,7 +2459,7 @@
       <c r="A68" s="4">
         <v>5</v>
       </c>
-      <c r="B68" s="14"/>
+      <c r="B68" s="17"/>
       <c r="C68" s="4">
         <v>10</v>
       </c>
@@ -2474,7 +2474,7 @@
       <c r="A69" s="4">
         <v>6</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="15" t="s">
         <v>80</v>
       </c>
       <c r="C69" s="4">
@@ -2491,7 +2491,7 @@
       <c r="A70" s="4">
         <v>6</v>
       </c>
-      <c r="B70" s="13"/>
+      <c r="B70" s="16"/>
       <c r="C70" s="4">
         <v>2</v>
       </c>
@@ -2506,7 +2506,7 @@
       <c r="A71" s="4">
         <v>6</v>
       </c>
-      <c r="B71" s="13"/>
+      <c r="B71" s="16"/>
       <c r="C71" s="4">
         <v>3</v>
       </c>
@@ -2521,7 +2521,7 @@
       <c r="A72" s="4">
         <v>6</v>
       </c>
-      <c r="B72" s="13"/>
+      <c r="B72" s="16"/>
       <c r="C72" s="4">
         <v>4</v>
       </c>
@@ -2536,7 +2536,7 @@
       <c r="A73" s="4">
         <v>6</v>
       </c>
-      <c r="B73" s="13"/>
+      <c r="B73" s="16"/>
       <c r="C73" s="4">
         <v>5</v>
       </c>
@@ -2551,7 +2551,7 @@
       <c r="A74" s="4">
         <v>6</v>
       </c>
-      <c r="B74" s="13"/>
+      <c r="B74" s="16"/>
       <c r="C74" s="4">
         <v>6</v>
       </c>
@@ -2566,7 +2566,7 @@
       <c r="A75" s="4">
         <v>6</v>
       </c>
-      <c r="B75" s="13"/>
+      <c r="B75" s="16"/>
       <c r="C75" s="4">
         <v>7</v>
       </c>
@@ -2581,7 +2581,7 @@
       <c r="A76" s="4">
         <v>6</v>
       </c>
-      <c r="B76" s="13"/>
+      <c r="B76" s="16"/>
       <c r="C76" s="4">
         <v>8</v>
       </c>
@@ -2596,7 +2596,7 @@
       <c r="A77" s="4">
         <v>6</v>
       </c>
-      <c r="B77" s="13"/>
+      <c r="B77" s="16"/>
       <c r="C77" s="4">
         <v>9</v>
       </c>
@@ -2611,7 +2611,7 @@
       <c r="A78" s="4">
         <v>6</v>
       </c>
-      <c r="B78" s="14"/>
+      <c r="B78" s="17"/>
       <c r="C78" s="4">
         <v>10</v>
       </c>
@@ -2626,7 +2626,7 @@
       <c r="A79" s="4">
         <v>7</v>
       </c>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="15" t="s">
         <v>91</v>
       </c>
       <c r="C79" s="4">
@@ -2643,7 +2643,7 @@
       <c r="A80" s="4">
         <v>7</v>
       </c>
-      <c r="B80" s="13"/>
+      <c r="B80" s="16"/>
       <c r="C80" s="4">
         <v>2</v>
       </c>
@@ -2658,7 +2658,7 @@
       <c r="A81" s="4">
         <v>7</v>
       </c>
-      <c r="B81" s="13"/>
+      <c r="B81" s="16"/>
       <c r="C81" s="4">
         <v>3</v>
       </c>
@@ -2673,7 +2673,7 @@
       <c r="A82" s="4">
         <v>7</v>
       </c>
-      <c r="B82" s="13"/>
+      <c r="B82" s="16"/>
       <c r="C82" s="4">
         <v>4</v>
       </c>
@@ -2688,7 +2688,7 @@
       <c r="A83" s="4">
         <v>7</v>
       </c>
-      <c r="B83" s="13"/>
+      <c r="B83" s="16"/>
       <c r="C83" s="4">
         <v>5</v>
       </c>
@@ -2703,7 +2703,7 @@
       <c r="A84" s="4">
         <v>7</v>
       </c>
-      <c r="B84" s="13"/>
+      <c r="B84" s="16"/>
       <c r="C84" s="4">
         <v>6</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="A85" s="4">
         <v>7</v>
       </c>
-      <c r="B85" s="13"/>
+      <c r="B85" s="16"/>
       <c r="C85" s="4">
         <v>7</v>
       </c>
@@ -2733,7 +2733,7 @@
       <c r="A86" s="4">
         <v>7</v>
       </c>
-      <c r="B86" s="13"/>
+      <c r="B86" s="16"/>
       <c r="C86" s="4">
         <v>8</v>
       </c>
@@ -2748,7 +2748,7 @@
       <c r="A87" s="4">
         <v>7</v>
       </c>
-      <c r="B87" s="13"/>
+      <c r="B87" s="16"/>
       <c r="C87" s="4">
         <v>9</v>
       </c>
@@ -2763,7 +2763,7 @@
       <c r="A88" s="4">
         <v>7</v>
       </c>
-      <c r="B88" s="13"/>
+      <c r="B88" s="16"/>
       <c r="C88" s="4">
         <v>10</v>
       </c>
@@ -2778,7 +2778,7 @@
       <c r="A89" s="4">
         <v>7</v>
       </c>
-      <c r="B89" s="14"/>
+      <c r="B89" s="17"/>
       <c r="C89" s="4">
         <v>11</v>
       </c>
@@ -2793,7 +2793,7 @@
       <c r="A90" s="4">
         <v>8</v>
       </c>
-      <c r="B90" s="12" t="s">
+      <c r="B90" s="15" t="s">
         <v>103</v>
       </c>
       <c r="C90" s="4">
@@ -2810,7 +2810,7 @@
       <c r="A91" s="4">
         <v>8</v>
       </c>
-      <c r="B91" s="13"/>
+      <c r="B91" s="16"/>
       <c r="C91" s="4">
         <v>2</v>
       </c>
@@ -2825,7 +2825,7 @@
       <c r="A92" s="4">
         <v>8</v>
       </c>
-      <c r="B92" s="13"/>
+      <c r="B92" s="16"/>
       <c r="C92" s="4">
         <v>3</v>
       </c>
@@ -2840,7 +2840,7 @@
       <c r="A93" s="4">
         <v>8</v>
       </c>
-      <c r="B93" s="13"/>
+      <c r="B93" s="16"/>
       <c r="C93" s="4">
         <v>4</v>
       </c>
@@ -2855,7 +2855,7 @@
       <c r="A94" s="4">
         <v>8</v>
       </c>
-      <c r="B94" s="13"/>
+      <c r="B94" s="16"/>
       <c r="C94" s="4">
         <v>5</v>
       </c>
@@ -2870,7 +2870,7 @@
       <c r="A95" s="4">
         <v>8</v>
       </c>
-      <c r="B95" s="13"/>
+      <c r="B95" s="16"/>
       <c r="C95" s="4">
         <v>6</v>
       </c>
@@ -2885,7 +2885,7 @@
       <c r="A96" s="4">
         <v>8</v>
       </c>
-      <c r="B96" s="13"/>
+      <c r="B96" s="16"/>
       <c r="C96" s="4">
         <v>7</v>
       </c>
@@ -2900,7 +2900,7 @@
       <c r="A97" s="4">
         <v>8</v>
       </c>
-      <c r="B97" s="13"/>
+      <c r="B97" s="16"/>
       <c r="C97" s="4">
         <v>8</v>
       </c>
@@ -2915,7 +2915,7 @@
       <c r="A98" s="4">
         <v>8</v>
       </c>
-      <c r="B98" s="13"/>
+      <c r="B98" s="16"/>
       <c r="C98" s="4">
         <v>9</v>
       </c>
@@ -2930,7 +2930,7 @@
       <c r="A99" s="4">
         <v>8</v>
       </c>
-      <c r="B99" s="13"/>
+      <c r="B99" s="16"/>
       <c r="C99" s="4">
         <v>10</v>
       </c>
@@ -2945,7 +2945,7 @@
       <c r="A100" s="4">
         <v>8</v>
       </c>
-      <c r="B100" s="13"/>
+      <c r="B100" s="16"/>
       <c r="C100" s="4">
         <v>11</v>
       </c>
@@ -2960,7 +2960,7 @@
       <c r="A101" s="4">
         <v>8</v>
       </c>
-      <c r="B101" s="14"/>
+      <c r="B101" s="17"/>
       <c r="C101" s="4">
         <v>12</v>
       </c>
@@ -4144,378 +4144,378 @@
   <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" style="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.33203125" style="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="149.33203125" style="15" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="15"/>
+    <col min="1" max="1" width="5" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="149.33203125" style="12" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="C1" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="16" t="s">
+      <c r="C1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="17">
+      <c r="A2" s="14">
         <v>6.1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D2" s="17"/>
+      <c r="D2" s="14"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="17">
+      <c r="A3" s="14">
         <v>6.2</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="14"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="17">
+      <c r="A4" s="14">
         <v>6.3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="14" t="s">
         <v>236</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D4" s="17"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="17">
+      <c r="A5" s="14">
         <v>6.4</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D5" s="17"/>
+      <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="17">
+      <c r="A6" s="14">
         <v>6.5</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D6" s="17"/>
+      <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="17">
+      <c r="A7" s="14">
         <v>6.6</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D7" s="17"/>
+      <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="17">
+      <c r="A8" s="14">
         <v>6.7</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D8" s="17"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="17">
+      <c r="A9" s="14">
         <v>6.8</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D9" s="17"/>
+      <c r="D9" s="14"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="17">
+      <c r="A10" s="14">
         <v>6.9</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D10" s="17"/>
+      <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+      <c r="A11" s="14">
         <v>6.1</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D11" s="17"/>
+      <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+      <c r="A12" s="14">
         <v>6.11</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D12" s="17"/>
+      <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="17">
+      <c r="A13" s="14">
         <v>6.12</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D13" s="17"/>
+      <c r="D13" s="14"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="17">
+      <c r="A14" s="14">
         <v>6.13</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D14" s="17"/>
+      <c r="D14" s="14"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="17">
+      <c r="A15" s="14">
         <v>6.14</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D15" s="17"/>
+      <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="17">
+      <c r="A16" s="14">
         <v>6.15</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D16" s="17"/>
+      <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="17">
+      <c r="A17" s="14">
         <v>6.16</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D17" s="17"/>
+      <c r="D17" s="14"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="17">
+      <c r="A18" s="14">
         <v>6.17</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="14" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="17">
+      <c r="A19" s="14">
         <v>6.18</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="14" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="17">
+      <c r="A20" s="14">
         <v>6.19</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="14" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="17">
+      <c r="A21" s="14">
         <v>6.2</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="14" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="17">
+      <c r="A22" s="14">
         <v>6.21</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="14" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="17">
+      <c r="A23" s="14">
         <v>6.22</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="14" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="17">
+      <c r="A24" s="14">
         <v>6.23</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="14" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="17">
+      <c r="A25" s="14">
         <v>6.24</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D25" s="17"/>
+      <c r="D25" s="14"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="17">
+      <c r="A26" s="14">
         <v>6.25</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D26" s="17"/>
+      <c r="D26" s="14"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="17">
+      <c r="A27" s="14">
         <v>6.26</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D27" s="17"/>
+      <c r="D27" s="14"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="17">
+      <c r="A28" s="14">
         <v>6.27</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="14" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="17">
+      <c r="A29" s="14">
         <v>6.28</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="D29" s="17"/>
+      <c r="D29" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
commit all the changes to branch
</commit_message>
<xml_diff>
--- a/Progress/Roadmap_progress.xlsx
+++ b/Progress/Roadmap_progress.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek\GIT Projects\MultiLinguinal_Application\Progress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF8D002-30BD-4D82-AB2A-0998B60DE824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE09ABB-4B93-4CBF-9E4B-E7C695540258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{B3A48A29-E4FC-423B-9095-878E848D4919}"/>
   </bookViews>
   <sheets>
     <sheet name="Road Map" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Road Map'!$A$1:$E$101</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="299">
   <si>
     <t>Step</t>
   </si>
@@ -907,6 +908,93 @@
 SELECT COUNT(*) FROM chat_app.messages;
 Exit:
 \q</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/auth</t>
+  </si>
+  <si>
+    <t>User Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/users</t>
+  </si>
+  <si>
+    <t>Language Configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/languages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/messages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/translations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/attachments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → features/sessions</t>
+  </si>
+  <si>
+    <t>WebSocket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → infrastructure/websocket</t>
+  </si>
+  <si>
+    <t>Redis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → infrastructure/redis</t>
+  </si>
+  <si>
+    <t>PostgreSQL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → infrastructure/database</t>
+  </si>
+  <si>
+    <t>Local File Storage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → infrastructure/storage</t>
+  </si>
+  <si>
+    <t>Encryption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → core/security + feature-specific usage</t>
+  </si>
+  <si>
+    <t>LangGraph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → ai/workflows</t>
+  </si>
+  <si>
+    <t>Agents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → ai/agents</t>
+  </si>
+  <si>
+    <t>Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → ai/tools</t>
+  </si>
+  <si>
+    <t>MCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    → ai/mcp</t>
   </si>
 </sst>
 </file>
@@ -4520,4 +4608,187 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D15CEF4-8592-4E21-B9F1-BB5DC007A5FD}">
+  <dimension ref="A1:A50"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="60.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>298</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>